<commit_message>
Save the Paul Lambda function library workbook.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/workbook/Paul Lambda function library.xlsx
+++ b/workbook/Paul Lambda function library.xlsx
@@ -10,7 +10,7 @@
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="8_{06C6CB15-630B-4D5E-8D9E-1C46BD761C74}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3120" yWindow="3120" windowWidth="21600" windowHeight="11295" xr2:uid="{F86E533F-AA82-4B92-9E31-B9766B011421}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{F86E533F-AA82-4B92-9E31-B9766B011421}"/>
   </bookViews>
   <sheets>
     <sheet name="Lambda functions" sheetId="2" r:id="rId1"/>
@@ -339,19 +339,19 @@
   <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
   </cellXfs>
@@ -372,6 +372,9 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
       <font>
         <b/>
         <i val="0"/>
@@ -389,9 +392,6 @@
         <scheme val="minor"/>
       </font>
     </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
@@ -406,7 +406,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{D86E44FA-9DA1-4E12-AC6D-519F6643549A}" name="tblLambdaFunctions" displayName="tblLambdaFunctions" ref="A6:C17" totalsRowShown="0" headerRowDxfId="3" dataDxfId="4">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{D86E44FA-9DA1-4E12-AC6D-519F6643549A}" name="tblLambdaFunctions" displayName="tblLambdaFunctions" ref="A6:C17" totalsRowShown="0" headerRowDxfId="4" dataDxfId="3">
   <autoFilter ref="A6:C17" xr:uid="{D86E44FA-9DA1-4E12-AC6D-519F6643549A}"/>
   <tableColumns count="3">
     <tableColumn id="1" xr3:uid="{9BC09484-693D-4D65-B451-5D7F46E9FE5C}" name="Name" dataDxfId="2"/>
@@ -743,32 +743,32 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:3" ht="24" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="2" t="s">
+      <c r="A1" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="2"/>
-      <c r="C1" s="2"/>
+      <c r="B1" s="5"/>
+      <c r="C1" s="5"/>
     </row>
     <row r="2" spans="1:3" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="3" t="s">
+      <c r="A2" s="6" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="3"/>
-      <c r="C2" s="3"/>
+      <c r="B2" s="6"/>
+      <c r="C2" s="6"/>
     </row>
     <row r="3" spans="1:3" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="3" t="s">
+      <c r="A3" s="6" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="3"/>
-      <c r="C3" s="3"/>
+      <c r="B3" s="6"/>
+      <c r="C3" s="6"/>
     </row>
     <row r="4" spans="1:3" ht="48" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="3" t="s">
+      <c r="A4" s="6" t="s">
         <v>3</v>
       </c>
-      <c r="B4" s="3"/>
-      <c r="C4" s="3"/>
+      <c r="B4" s="6"/>
+      <c r="C4" s="6"/>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
@@ -781,124 +781,124 @@
         <v>6</v>
       </c>
     </row>
-    <row r="7" spans="1:3" s="5" customFormat="1" ht="150" x14ac:dyDescent="0.25">
-      <c r="A7" s="4" t="s">
+    <row r="7" spans="1:3" s="2" customFormat="1" ht="150" x14ac:dyDescent="0.25">
+      <c r="A7" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="B7" s="4" t="s">
+      <c r="B7" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="C7" s="4" t="s">
+      <c r="C7" s="3" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="8" spans="1:3" s="5" customFormat="1" ht="30" x14ac:dyDescent="0.25">
-      <c r="A8" s="4" t="s">
+    <row r="8" spans="1:3" s="2" customFormat="1" ht="30" x14ac:dyDescent="0.25">
+      <c r="A8" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="B8" s="4" t="s">
+      <c r="B8" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="C8" s="4" t="s">
+      <c r="C8" s="3" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="9" spans="1:3" s="5" customFormat="1" ht="75" x14ac:dyDescent="0.25">
-      <c r="A9" s="4" t="s">
+    <row r="9" spans="1:3" s="2" customFormat="1" ht="75" x14ac:dyDescent="0.25">
+      <c r="A9" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="B9" s="4" t="s">
+      <c r="B9" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="C9" s="4" t="s">
+      <c r="C9" s="3" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="10" spans="1:3" s="5" customFormat="1" ht="45" x14ac:dyDescent="0.25">
-      <c r="A10" s="4" t="s">
+    <row r="10" spans="1:3" s="2" customFormat="1" ht="45" x14ac:dyDescent="0.25">
+      <c r="A10" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="B10" s="4" t="s">
+      <c r="B10" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="C10" s="4" t="s">
+      <c r="C10" s="3" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="11" spans="1:3" s="5" customFormat="1" ht="30" x14ac:dyDescent="0.25">
-      <c r="A11" s="4" t="s">
+    <row r="11" spans="1:3" s="2" customFormat="1" ht="30" x14ac:dyDescent="0.25">
+      <c r="A11" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="B11" s="4" t="s">
+      <c r="B11" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="C11" s="4" t="s">
+      <c r="C11" s="3" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="12" spans="1:3" s="5" customFormat="1" ht="45" x14ac:dyDescent="0.25">
-      <c r="A12" s="4" t="s">
+    <row r="12" spans="1:3" s="2" customFormat="1" ht="45" x14ac:dyDescent="0.25">
+      <c r="A12" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="B12" s="4" t="s">
+      <c r="B12" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="C12" s="4" t="s">
+      <c r="C12" s="3" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="13" spans="1:3" s="5" customFormat="1" ht="45" x14ac:dyDescent="0.25">
-      <c r="A13" s="4" t="s">
+    <row r="13" spans="1:3" s="2" customFormat="1" ht="45" x14ac:dyDescent="0.25">
+      <c r="A13" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="B13" s="4" t="s">
+      <c r="B13" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="C13" s="4" t="s">
+      <c r="C13" s="3" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="14" spans="1:3" s="5" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="4" t="s">
+    <row r="14" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="B14" s="4" t="s">
+      <c r="B14" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="C14" s="4" t="s">
+      <c r="C14" s="3" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="15" spans="1:3" s="5" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="4" t="s">
+    <row r="15" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A15" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="B15" s="4" t="s">
+      <c r="B15" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="C15" s="4" t="s">
+      <c r="C15" s="3" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="16" spans="1:3" s="5" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="4" t="s">
+    <row r="16" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="3" t="s">
         <v>34</v>
       </c>
-      <c r="B16" s="4" t="s">
+      <c r="B16" s="3" t="s">
         <v>35</v>
       </c>
-      <c r="C16" s="4" t="s">
+      <c r="C16" s="3" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="17" spans="1:3" s="5" customFormat="1" ht="120" x14ac:dyDescent="0.25">
-      <c r="A17" s="4" t="s">
+    <row r="17" spans="1:3" s="2" customFormat="1" ht="120" x14ac:dyDescent="0.25">
+      <c r="A17" s="3" t="s">
         <v>37</v>
       </c>
-      <c r="B17" s="4" t="s">
+      <c r="B17" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="C17" s="4" t="s">
+      <c r="C17" s="3" t="s">
         <v>39</v>
       </c>
     </row>
@@ -925,12 +925,12 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:1" ht="36" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="6" t="s">
+      <c r="A1" s="4" t="s">
         <v>40</v>
       </c>
     </row>
     <row r="2" spans="1:1" ht="399.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="4" t="s">
+      <c r="A2" s="3" t="s">
         <v>41</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Update the Paul Lambda function library workbook.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/workbook/Paul Lambda function library.xlsx
+++ b/workbook/Paul Lambda function library.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/77eae79058c0e1af/Notebooks/Cursor/Excel-OfficeScripts-Library/workbook/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{06C6CB15-630B-4D5E-8D9E-1C46BD761C74}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="52" documentId="8_{06C6CB15-630B-4D5E-8D9E-1C46BD761C74}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{248A6C4D-B758-46D1-B957-8EFAF082895E}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{F86E533F-AA82-4B92-9E31-B9766B011421}"/>
   </bookViews>
@@ -16,6 +16,19 @@
     <sheet name="Lambda functions" sheetId="2" r:id="rId1"/>
     <sheet name="Activate script" sheetId="1" r:id="rId2"/>
   </sheets>
+  <definedNames>
+    <definedName name="DDL" comment="Dependent drop-down list from a hierarchy table. With no lookups, returns column 1; otherwise returns the next-level values that match the parent path.">_xlfn.LAMBDA(_xlpm.range,_xlop.lookup1,_xlop.lookup2,_xlop.lookup3,_xlop.lookup4,_xlop.lookup5,_xlop.lookup6,_xlop.lookup7,_xlop.lookup8,_xlop.lookup9,_xlop.lookup10,_xlfn.LET(_xlpm._s, "%^&amp;&amp;@", _xlpm.lookupValue, _xlpm.lookup1 &amp; _xlpm._s &amp; _xlpm.lookup2 &amp; _xlpm._s &amp; _xlpm.lookup3 &amp; _xlpm._s &amp; _xlpm.lookup4 &amp; _xlpm._s &amp; _xlpm.lookup5 &amp; _xlpm._s &amp; _xlpm.lookup6 &amp; _xlpm._s &amp; _xlpm.lookup7 &amp; _xlpm._s &amp; _xlpm.lookup8 &amp; _xlpm._s &amp; _xlpm.lookup9 &amp; _xlpm._s &amp; _xlpm.lookup10, _xlpm.levelIndex, IFERROR(ROWS(_xlfn.TEXTSPLIT(_xlpm.lookupValue, , _xlpm._s, TRUE())), 0) + 1, _xlpm.lookupArray, _xlfn.BYROW(_xlfn.EXPAND(_xlfn.CHOOSECOLS(_xlpm.range, _xlfn.SEQUENCE(1, _xlpm.levelIndex - 1)), , 10, ""), _xlfn.LAMBDA(_xlpm.row, _xlfn.TEXTJOIN(_xlpm._s, FALSE, _xlpm.row))), _xlpm.returnRange, INDEX(_xlpm.range, 0, _xlpm.levelIndex), _xlpm.result, IF(_xlfn.ISOMITTED(_xlpm.lookup1) * _xlpm.levelIndex = 1, _xlpm.returnRange, _xlfn.XLOOKUP(_xlpm.lookupValue, _xlpm.lookupArray, _xlpm.returnRange):_xlfn.XLOOKUP(_xlpm.lookupValue, _xlpm.lookupArray, _xlpm.returnRange, , , -1)), _xlpm.result))</definedName>
+    <definedName name="DDLSorter" comment="Sort a hierarchy table by every column left to right so identical parent paths are contiguous for DDL.">_xlfn.LAMBDA(_xlpm.Range,_xlop.SortOrder,_xlfn._xlws.SORT(_xlpm.Range, _xlfn.SEQUENCE(, COLUMNS(_xlpm.Range)), _xlpm.SortOrder))</definedName>
+    <definedName name="DoubleXLookup" comment="Two-way lookup: XMATCH the row header and column header, then INDEX into the body. Optional if_not_found and XMATCH modes.">_xlfn.LAMBDA(_xlpm.vlookup_value,_xlpm.vlookup_array,_xlpm.hlookup_value,_xlpm.hlookup_array,_xlpm.return_array,_xlop.if_not_found,_xlop.vmatch_mode,_xlop.vsearch_mode,_xlop.hmatch_mode,_xlop.hsearch_mode, IFERROR( INDEX(_xlpm.return_array,_xlfn.XMATCH(_xlpm.vlookup_value,_xlpm.vlookup_array,_xlpm.vmatch_mode,_xlpm.vsearch_mode),_xlfn.XMATCH(_xlpm.hlookup_value,_xlpm.hlookup_array,_xlpm.hmatch_mode,_xlpm.hsearch_mode)), IF(_xlfn.ISOMITTED(_xlpm.if_not_found),NA(),_xlpm.if_not_found)))</definedName>
+    <definedName name="ESMOOTHWEIGHTEDVALUES" comment="Each value times its exponential-smoothing weight (default alpha 0.2). Weights are the same as EXPSMOOTHWEIGHTS.">_xlfn.LAMBDA(_xlpm.values,_xlop.alpha,_xlfn.LET(_xlpm.a,IF(_xlfn.ISOMITTED(_xlpm.alpha),0.2,_xlpm.alpha),_xlpm.n,ROWS(_xlpm.values),_xlpm.w,_xlpm.a*(1-_xlpm.a)^(_xlpm.n-_xlfn.SEQUENCE(_xlpm.n)),_xlpm.residual,1-SUM(_xlpm.w),_xlpm.adjW,_xlpm.w+(_xlfn.SEQUENCE(_xlpm.n)=1)*_xlpm.residual,_xlpm.values*_xlpm.adjW))</definedName>
+    <definedName name="EXPSMOOTH" comment="Simple exponential smoothing of a column (default alpha 0.2). Returns only the last smoothed value.">_xlfn.LAMBDA(_xlpm.data,_xlop.alpha,_xlfn.LET(_xlpm.a,IF(_xlfn.ISOMITTED(_xlpm.alpha),0.2,_xlpm.alpha),_xlpm.smooth,_xlfn.SCAN(INDEX(_xlpm.data,1),_xlfn.DROP(_xlpm.data,1),_xlfn.LAMBDA(_xlpm.prev,_xlpm.x,_xlpm.a*_xlpm.x+(1-_xlpm.a)*_xlpm.prev)),_xlfn.TAKE(_xlpm.smooth,-1)))</definedName>
+    <definedName name="EXPSMOOTHSERIES" comment="Simple exponential smoothing of a column (default alpha 0.2). Returns the full series, starting with the first observation.">_xlfn.LAMBDA(_xlpm.data,_xlop.alpha,_xlfn.LET(_xlpm.a,IF(_xlfn.ISOMITTED(_xlpm.alpha),0.2,_xlpm.alpha),_xlfn.VSTACK(INDEX(_xlpm.data,1),_xlfn.SCAN(INDEX(_xlpm.data,1),_xlfn.DROP(_xlpm.data,1),_xlfn.LAMBDA(_xlpm.prev,_xlpm.x,_xlpm.a*_xlpm.x+(1-_xlpm.a)*_xlpm.prev)))))</definedName>
+    <definedName name="EXPSMOOTHWEIGHTS" comment="Exponential-smoothing weights for a column, default alpha 0.2. Residual mass is added to the first weight so they sum to 1.">_xlfn.LAMBDA(_xlpm.values,_xlop.alpha,_xlfn.LET(_xlpm.a,IF(_xlfn.ISOMITTED(_xlpm.alpha),0.2,_xlpm.alpha),_xlpm.n,ROWS(_xlpm.values),_xlpm.w,_xlpm.a*(1-_xlpm.a)^(_xlpm.n-_xlfn.SEQUENCE(_xlpm.n)),_xlpm.residual,1-SUM(_xlpm.w),_xlpm.w+(_xlfn.SEQUENCE(_xlpm.n)=1)*_xlpm.residual))</definedName>
+    <definedName name="IFERROR0" comment="Return the value, or 0 if the value is an error.">_xlfn.LAMBDA(_xlpm.value, IFERROR(_xlpm.value, 0))</definedName>
+    <definedName name="ISZERO2" comment="TRUE if a number rounds to zero at two decimal places.">_xlfn.LAMBDA(_xlpm.value, ROUND(_xlpm.value, 2)=0)</definedName>
+    <definedName name="ROUND2" comment="Round a number to two decimal places.">_xlfn.LAMBDA(_xlpm.value, ROUND(_xlpm.value, 2))</definedName>
+    <definedName name="SuperXLookup" comment="XLOOKUP that returns a whole row or whole column. One-column lookup_value matches a row; otherwise it matches a column.">_xlfn.LAMBDA(_xlpm.lookup_value,_xlpm.lookup_array,_xlpm.return_array,_xlop.if_not_found,_xlop.match_mode,_xlop.search_mode, IF(COLUMNS(_xlpm.lookup_value)=1, IFERROR(INDEX(_xlpm.return_array,_xlfn.XMATCH(_xlpm.lookup_value,_xlpm.lookup_array,_xlpm.match_mode,_xlpm.search_mode),_xlfn.SEQUENCE(1,COLUMNS(_xlpm.return_array))),IF(_xlfn.ISOMITTED(_xlpm.if_not_found),NA(),_xlpm.if_not_found)), IFERROR(INDEX(_xlpm.return_array,_xlfn.SEQUENCE(ROWS(_xlpm.return_array)),_xlfn.XMATCH(_xlpm.lookup_value,_xlpm.lookup_array,_xlpm.match_mode,_xlpm.search_mode)),IF(_xlfn.ISOMITTED(_xlpm.if_not_found),NA(),_xlpm.if_not_found))))</definedName>
+  </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -39,6 +52,43 @@
 </workbook>
 </file>
 
+<file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+  <metadataTypes count="2">
+    <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
+    <metadataType name="XLRICHVALUE" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1"/>
+  </metadataTypes>
+  <futureMetadata name="XLDAPR" count="1">
+    <bk>
+      <extLst>
+        <ext uri="{bdbb8cdc-fa1e-496e-a857-3c3f30c029c3}">
+          <xda:dynamicArrayProperties fDynamic="1" fCollapsed="0"/>
+        </ext>
+      </extLst>
+    </bk>
+  </futureMetadata>
+  <futureMetadata name="XLRICHVALUE" count="1">
+    <bk>
+      <extLst>
+        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
+          <xlrd:rvb i="0"/>
+        </ext>
+      </extLst>
+    </bk>
+  </futureMetadata>
+  <cellMetadata count="1">
+    <bk>
+      <rc t="1" v="0"/>
+    </bk>
+  </cellMetadata>
+  <valueMetadata count="1">
+    <bk>
+      <rc t="2" v="0"/>
+    </bk>
+  </valueMetadata>
+</metadata>
+</file>
+
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="42">
   <si>
@@ -165,125 +215,112 @@
     <t>Paste this into Automate -&gt; New Script. Save as Activate Lambda functions. Then use sheet Lambda functions.</t>
   </si>
   <si>
-    <t xml:space="preserve">/**_x000D_
- * Activate Lambda functions_x000D_
- *_x000D_
- * On sheet **Lambda functions**, select one or more table rows and Run._x000D_
- * Each selected Name is written to this workbook's Name Manager_x000D_
- * (replaced if it already exists) using the Lambda code column._x000D_
- *_x000D_
- * Automate â†’ New Script â†’ paste this file â†’ Save as **Activate Lambda functions**._x000D_
- */_x000D_
-function main(workbook: ExcelScript.Workbook): void {_x000D_
-  const sheetName = "Lambda functions";_x000D_
-  const sheet = workbook.getWorksheet(sheetName);_x000D_
-  if (!sheet) {_x000D_
-    throw new Error('Sheet "Lambda functions" was not found.');_x000D_
-  }_x000D_
-_x000D_
-  const selected = workbook.getSelectedRange();_x000D_
-  if (selected.getWorksheet().getName() !== sheetName) {_x000D_
-    throw new Error('Select one or more rows on "Lambda functions", then run this script.');_x000D_
-  }_x000D_
-_x000D_
-  const headerRow = findHeaderRow(sheet);_x000D_
-  if (headerRow &lt; 0) {_x000D_
-    throw new Error('Could not find a header row with Name, Lambda code, Note.');_x000D_
-  }_x000D_
-_x000D_
-  const first = selected.getRowIndex();_x000D_
-  const rowCount = selected.getRowCount();_x000D_
-  let activated = 0;_x000D_
-  const skipped: string[] = [];_x000D_
-_x000D_
-  for (let i = 0; i &lt; rowCount; i++) {_x000D_
-    const row = first + i;_x000D_
-    if (row &lt;= headerRow) {_x000D_
-      continue;_x000D_
-    }_x000D_
-_x000D_
-    const name = cellText(sheet, row, 0);_x000D_
-    const formula = lambdaFormula(sheet, row, 1);_x000D_
-    const note = cellText(sheet, row, 2);_x000D_
-_x000D_
-    if (name === "" || name === "Name") {_x000D_
-      continue;_x000D_
-    }_x000D_
-    if (formula === "") {_x000D_
-      skipped.push(name + " (no Lambda code)");_x000D_
-      continue;_x000D_
-    }_x000D_
-_x000D_
-    replaceNamedItem(workbook, name, formula, note);_x000D_
-    activated++;_x000D_
-  }_x000D_
-_x000D_
-  if (activated === 0) {_x000D_
-    throw new Error('No function rows were selected. Select rows under the Name / Lambda code / Note header.');_x000D_
-  }_x000D_
-_x000D_
-  console.log("Activated " + activated + " named function(s) in Name Manager.");_x000D_
-  if (skipped.length &gt; 0) {_x000D_
-    console.log("Skipped: " + skipped.join("; "));_x000D_
-  }_x000D_
-}_x000D_
-_x000D_
-function findHeaderRow(sheet: ExcelScript.Worksheet): number {_x000D_
-  for (let r = 0; r &lt; 20; r++) {_x000D_
-    const a = cellText(sheet, r, 0).toLowerCase();_x000D_
-    const b = cellText(sheet, r, 1).toLowerCase();_x000D_
-    if (a === "name" &amp;&amp; b.indexOf("lambda") &gt;= 0) {_x000D_
-      return r;_x000D_
-    }_x000D_
-  }_x000D_
-  return -1;_x000D_
-}_x000D_
-_x000D_
-function cellText(sheet: ExcelScript.Worksheet, row: number, column: number): string {_x000D_
-  const cell = sheet.getCell(row, column);_x000D_
-  const value = cell.getValue();_x000D_
-  if (value === undefined || value === null) {_x000D_
-    return "";_x000D_
-  }_x000D_
-  return String(value).trim();_x000D_
-}_x000D_
-_x000D_
-function lambdaFormula(sheet: ExcelScript.Worksheet, row: number, column: number): string {_x000D_
-  const cell = sheet.getCell(row, column);_x000D_
-  let formula = "";_x000D_
-  const asFormula = cell.getFormula();_x000D_
-  if (asFormula &amp;&amp; String(asFormula).charAt(0) === "=") {_x000D_
-    formula = String(asFormula).trim();_x000D_
-  } else {_x000D_
-    formula = cellText(sheet, row, column);_x000D_
-  }_x000D_
-  if (formula.charAt(0) === "'") {_x000D_
-    formula = formula.substring(1);_x000D_
-  }_x000D_
-  if (formula !== "" &amp;&amp; formula.charAt(0) !== "=") {_x000D_
-    formula = "=" + formula;_x000D_
-  }_x000D_
-  return formula;_x000D_
-}_x000D_
-_x000D_
-function replaceNamedItem(_x000D_
-  workbook: ExcelScript.Workbook,_x000D_
-  name: string,_x000D_
-  formula: string,_x000D_
-  note: string_x000D_
-): void {_x000D_
-  const items = workbook.getNamedItems();_x000D_
-  for (let i = 0; i &lt; items.length; i++) {_x000D_
-    if (items[i].getName() === name) {_x000D_
-      items[i].delete();_x000D_
-      break;_x000D_
-    }_x000D_
-  }_x000D_
-  const item = workbook.addNamedItem(name, formula);_x000D_
-  if (note &amp;&amp; note !== "") {_x000D_
-    item.setComment(note);_x000D_
-  }_x000D_
-}_x000D_
+    <t xml:space="preserve">/**
+ * Activate Lambda functions
+ *
+ * On sheet **Lambda functions**, select one or more table rows and Run.
+ * Each selected Name is written to this workbook's Name Manager
+ * (replaced if it already exists) using the Lambda code column.
+ *
+ * Automate â†’ New Script â†’ paste this file â†’ Save as **Activate Lambda functions**.
+ */
+function main(workbook: ExcelScript.Workbook): void {
+  const sheetName = "Lambda functions";
+  const sheet = workbook.getWorksheet(sheetName);
+  if (!sheet) {
+    throw new Error('Sheet "Lambda functions" was not found.');
+  }
+  const selected = workbook.getSelectedRange();
+  if (selected.getWorksheet().getName() !== sheetName) {
+    throw new Error('Select one or more rows on "Lambda functions", then run this script.');
+  }
+  const headerRow = findHeaderRow(sheet);
+  if (headerRow &lt; 0) {
+    throw new Error('Could not find a header row with Name, Lambda code, Note.');
+  }
+  const first = selected.getRowIndex();
+  const rowCount = selected.getRowCount();
+  let activated = 0;
+  const skipped: string[] = [];
+  for (let i = 0; i &lt; rowCount; i++) {
+    const row = first + i;
+    if (row &lt;= headerRow) {
+      continue;
+    }
+    const name = cellText(sheet, row, 0);
+    const formula = lambdaFormula(sheet, row, 1);
+    const note = cellText(sheet, row, 2);
+    if (name === "" || name === "Name") {
+      continue;
+    }
+    if (formula === "") {
+      skipped.push(name + " (no Lambda code)");
+      continue;
+    }
+    replaceNamedItem(workbook, name, formula, note);
+    activated++;
+  }
+  if (activated === 0) {
+    throw new Error('No function rows were selected. Select rows under the Name / Lambda code / Note header.');
+  }
+  console.log("Activated " + activated + " named function(s) in Name Manager.");
+  if (skipped.length &gt; 0) {
+    console.log("Skipped: " + skipped.join("; "));
+  }
+}
+function findHeaderRow(sheet: ExcelScript.Worksheet): number {
+  for (let r = 0; r &lt; 20; r++) {
+    const a = cellText(sheet, r, 0).toLowerCase();
+    const b = cellText(sheet, r, 1).toLowerCase();
+    if (a === "name" &amp;&amp; b.indexOf("lambda") &gt;= 0) {
+      return r;
+    }
+  }
+  return -1;
+}
+function cellText(sheet: ExcelScript.Worksheet, row: number, column: number): string {
+  const cell = sheet.getCell(row, column);
+  const value = cell.getValue();
+  if (value === undefined || value === null) {
+    return "";
+  }
+  return String(value).trim();
+}
+function lambdaFormula(sheet: ExcelScript.Worksheet, row: number, column: number): string {
+  const cell = sheet.getCell(row, column);
+  let formula = "";
+  const asFormula = cell.getFormula();
+  if (asFormula &amp;&amp; String(asFormula).charAt(0) === "=") {
+    formula = String(asFormula).trim();
+  } else {
+    formula = cellText(sheet, row, column);
+  }
+  if (formula.charAt(0) === "'") {
+    formula = formula.substring(1);
+  }
+  if (formula !== "" &amp;&amp; formula.charAt(0) !== "=") {
+    formula = "=" + formula;
+  }
+  return formula;
+}
+function replaceNamedItem(
+  workbook: ExcelScript.Workbook,
+  name: string,
+  formula: string,
+  note: string
+): void {
+  const items = workbook.getNamedItems();
+  for (let i = 0; i &lt; items.length; i++) {
+    if (items[i].getName() === name) {
+      items[i].delete();
+      break;
+    }
+  }
+  const item = workbook.addNamedItem(name, formula);
+  if (note &amp;&amp; note !== "") {
+    item.setComment(note);
+  }
+}
 </t>
   </si>
 </sst>
@@ -403,6 +440,70 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
+</file>
+
+<file path=xl/richData/rdRichValueTypes.xml><?xml version="1.0" encoding="utf-8"?>
+<rvTypesInfo xmlns="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" mc:Ignorable="x">
+  <global>
+    <keyFlags>
+      <key name="_Self">
+        <flag name="ExcludeFromFile" value="1"/>
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_DisplayString">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_Flags">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_Format">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_SubLabel">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_Attribution">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_Icon">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_Display">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_CanonicalPropertyNames">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_ClassificationId">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+    </keyFlags>
+  </global>
+</rvTypesInfo>
+</file>
+
+<file path=xl/richData/rdrichvalue.xml><?xml version="1.0" encoding="utf-8"?>
+<rvData xmlns="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" count="1">
+  <rv s="0">
+    <v>2</v>
+    <v>6</v>
+    <v>19</v>
+  </rv>
+</rvData>
+</file>
+
+<file path=xl/richData/rdrichvaluestructure.xml><?xml version="1.0" encoding="utf-8"?>
+<rvStructures xmlns="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" count="1">
+  <s t="_error">
+    <k n="errorType" t="i"/>
+    <k n="argument" t="s"/>
+    <k n="subType" t="i"/>
+  </s>
+</rvStructures>
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -734,7 +835,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2755F84D-CD28-4166-9AB8-1A2E95AA3384}">
-  <dimension ref="A1:C17"/>
+  <dimension ref="A1:C22"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="28.7109375" customWidth="1"/>
@@ -900,6 +1001,12 @@
       </c>
       <c r="C17" s="3" t="s">
         <v>39</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A22" t="e" cm="1" vm="1">
+        <f t="array" ref="A22">SuperXLookup()</f>
+        <v>#VALUE!</v>
       </c>
     </row>
   </sheetData>

</xml_diff>